<commit_message>
Alle 5 store ligaer er færdige, jeg har opdateret LightGBM modellen og jeg har eksperimenteret med alternative modeller
</commit_message>
<xml_diff>
--- a/English Premier League/Træning og forudsigelse/X_pred.xlsx
+++ b/English Premier League/Træning og forudsigelse/X_pred.xlsx
@@ -6253,37 +6253,37 @@
         <v>1</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O9" t="n">
         <v>1</v>
@@ -6295,10 +6295,10 @@
         <v>0</v>
       </c>
       <c r="R9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T9" t="n">
         <v>1</v>
@@ -6307,28 +6307,28 @@
         <v>1</v>
       </c>
       <c r="V9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X9" t="n">
         <v>0</v>
       </c>
       <c r="Y9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Z9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AA9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB9" t="n">
         <v>1</v>
       </c>
       <c r="AC9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AD9" t="n">
         <v>0</v>
@@ -6337,10 +6337,10 @@
         <v>1</v>
       </c>
       <c r="AF9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AH9" t="n">
         <v>0</v>
@@ -6352,13 +6352,13 @@
         <v>0</v>
       </c>
       <c r="AK9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AL9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AM9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AN9" t="n">
         <v>1</v>
@@ -6370,7 +6370,7 @@
         <v>0</v>
       </c>
       <c r="AQ9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR9" t="n">
         <v>0</v>
@@ -6379,7 +6379,7 @@
         <v>1</v>
       </c>
       <c r="AT9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU9" t="n">
         <v>0</v>
@@ -6397,25 +6397,25 @@
         <v>0</v>
       </c>
       <c r="AZ9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BA9" t="n">
         <v>0</v>
       </c>
       <c r="BB9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BD9" t="n">
         <v>0</v>
       </c>
       <c r="BE9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BF9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG9" t="n">
         <v>0</v>
@@ -6424,7 +6424,7 @@
         <v>1</v>
       </c>
       <c r="BI9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BJ9" t="n">
         <v>1</v>
@@ -6436,100 +6436,100 @@
         <v>0</v>
       </c>
       <c r="BM9" t="n">
-        <v>3.137931034482758</v>
+        <v>3.103448275862069</v>
       </c>
       <c r="BN9" t="n">
-        <v>3.631448275862069</v>
+        <v>3.222620689655172</v>
       </c>
       <c r="BO9" t="n">
-        <v>30.86731034482758</v>
+        <v>25.24386206896552</v>
       </c>
       <c r="BP9" t="n">
-        <v>9.683862068965517</v>
+        <v>9.667862068965517</v>
       </c>
       <c r="BQ9" t="n">
-        <v>158.5732413793103</v>
+        <v>117.0885517241379</v>
       </c>
       <c r="BR9" t="n">
-        <v>29.6568275862069</v>
+        <v>31.68910344827586</v>
       </c>
       <c r="BS9" t="n">
-        <v>18.76248275862069</v>
+        <v>10.20496551724138</v>
       </c>
       <c r="BT9" t="n">
-        <v>84.12855172413794</v>
+        <v>40.28275862068966</v>
       </c>
       <c r="BU9" t="n">
-        <v>1840.539034482759</v>
+        <v>1354.574896551724</v>
       </c>
       <c r="BV9" t="n">
-        <v>54.47172413793103</v>
+        <v>48.87641379310345</v>
       </c>
       <c r="BW9" t="n">
-        <v>27.23586206896552</v>
+        <v>16.65020689655172</v>
       </c>
       <c r="BX9" t="n">
-        <v>41.15641379310345</v>
+        <v>44.57958620689655</v>
       </c>
       <c r="BY9" t="n">
-        <v>75.04993103448277</v>
+        <v>80.56551724137931</v>
       </c>
       <c r="BZ9" t="n">
-        <v>6.657655172413794</v>
+        <v>2.68551724137931</v>
       </c>
       <c r="CA9" t="n">
-        <v>19.97296551724138</v>
+        <v>20.40993103448276</v>
       </c>
       <c r="CB9" t="n">
-        <v>59.91889655172414</v>
+        <v>45.65379310344827</v>
       </c>
       <c r="CC9" t="n">
-        <v>185.8091034482759</v>
+        <v>172.9473103448276</v>
       </c>
       <c r="CD9" t="n">
-        <v>1503.419586206897</v>
+        <v>1017.273931034483</v>
       </c>
       <c r="CE9" t="n">
-        <v>1197.167448275862</v>
+        <v>778.8</v>
       </c>
       <c r="CF9" t="n">
-        <v>239.6755862068966</v>
+        <v>202.488</v>
       </c>
       <c r="CG9" t="n">
-        <v>0.353363148728666</v>
+        <v>0.3576099027409372</v>
       </c>
       <c r="CH9" t="n">
-        <v>0.9310935562521769</v>
+        <v>1.011315296198055</v>
       </c>
       <c r="CI9" t="n">
-        <v>0.4466711947056775</v>
+        <v>0.3746839080459771</v>
       </c>
       <c r="CJ9" t="n">
-        <v>1.213157436433298</v>
+        <v>0.8189989858012171</v>
       </c>
       <c r="CK9" t="n">
-        <v>0.1698863221429156</v>
+        <v>0.1115022829152983</v>
       </c>
       <c r="CL9" t="n">
-        <v>0.3867345132920047</v>
+        <v>0.4904317083368588</v>
       </c>
       <c r="CM9" t="n">
-        <v>2.396755862068966</v>
+        <v>2.02488</v>
       </c>
       <c r="CN9" t="n">
-        <v>1.516292237698098</v>
+        <v>1.225015353037767</v>
       </c>
       <c r="CO9" t="n">
-        <v>0.1781171806554555</v>
+        <v>0.1311755543639581</v>
       </c>
       <c r="CP9" t="n">
-        <v>1.59110656255598</v>
+        <v>1.169841425939701</v>
       </c>
       <c r="CQ9" t="n">
-        <v>1.575395725678927</v>
+        <v>1.22430269357164</v>
       </c>
       <c r="CR9" t="n">
-        <v>0.2088584651740999</v>
+        <v>0.1388317490293456</v>
       </c>
       <c r="CS9" t="n">
         <v>1</v>
@@ -6538,10 +6538,10 @@
         <v>0</v>
       </c>
       <c r="CU9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CV9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="CW9" t="n">
         <v>0</v>
@@ -6556,19 +6556,19 @@
         <v>1</v>
       </c>
       <c r="DA9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DB9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DC9" t="n">
         <v>1</v>
       </c>
       <c r="DD9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DE9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DF9" t="n">
         <v>1</v>
@@ -6580,19 +6580,19 @@
         <v>1</v>
       </c>
       <c r="DI9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DJ9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DK9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DL9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="DM9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DN9" t="n">
         <v>0</v>
@@ -6601,19 +6601,19 @@
         <v>0</v>
       </c>
       <c r="DP9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DQ9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DR9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DS9" t="n">
         <v>1</v>
       </c>
       <c r="DT9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="DU9" t="n">
         <v>0</v>
@@ -6634,10 +6634,10 @@
         <v>0</v>
       </c>
       <c r="EA9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="EB9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="EC9" t="n">
         <v>1</v>
@@ -6658,10 +6658,10 @@
         <v>1</v>
       </c>
       <c r="EI9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="EJ9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="EK9" t="n">
         <v>0</v>
@@ -6673,19 +6673,19 @@
         <v>1</v>
       </c>
       <c r="EN9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="EO9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="EP9" t="n">
         <v>0</v>
       </c>
       <c r="EQ9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ER9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="ES9" t="n">
         <v>1</v>
@@ -6703,7 +6703,7 @@
         <v>0</v>
       </c>
       <c r="EX9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="EY9" t="n">
         <v>0</v>
@@ -6712,205 +6712,205 @@
         <v>1</v>
       </c>
       <c r="FA9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="FB9" t="n">
         <v>1</v>
       </c>
       <c r="FC9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="FD9" t="n">
         <v>0</v>
       </c>
       <c r="FE9" t="n">
-        <v>2.475862068965517</v>
+        <v>3.793103448275862</v>
       </c>
       <c r="FF9" t="n">
-        <v>4.146758620689655</v>
+        <v>5.33544827586207</v>
       </c>
       <c r="FG9" t="n">
-        <v>31.61903448275861</v>
+        <v>35.5696551724138</v>
       </c>
       <c r="FH9" t="n">
-        <v>12.95862068965517</v>
+        <v>11.26372413793103</v>
       </c>
       <c r="FI9" t="n">
-        <v>137.3613793103448</v>
+        <v>164.8060689655173</v>
       </c>
       <c r="FJ9" t="n">
-        <v>23.84386206896551</v>
+        <v>30.82703448275862</v>
       </c>
       <c r="FK9" t="n">
-        <v>15.032</v>
+        <v>19.56331034482758</v>
       </c>
       <c r="FL9" t="n">
-        <v>50.27944827586205</v>
+        <v>48.01903448275862</v>
       </c>
       <c r="FM9" t="n">
-        <v>1689.804137931034</v>
+        <v>1876.892137931035</v>
       </c>
       <c r="FN9" t="n">
-        <v>43.02262068965516</v>
+        <v>49.79751724137932</v>
       </c>
       <c r="FO9" t="n">
-        <v>17.10537931034482</v>
+        <v>24.89875862068966</v>
       </c>
       <c r="FP9" t="n">
-        <v>38.35751724137931</v>
+        <v>39.71944827586207</v>
       </c>
       <c r="FQ9" t="n">
-        <v>77.23337931034482</v>
+        <v>65.80386206896551</v>
       </c>
       <c r="FR9" t="n">
-        <v>2.591724137931034</v>
+        <v>5.33544827586207</v>
       </c>
       <c r="FS9" t="n">
-        <v>16.58703448275862</v>
+        <v>18.97048275862069</v>
       </c>
       <c r="FT9" t="n">
-        <v>48.72441379310344</v>
+        <v>50.39034482758621</v>
       </c>
       <c r="FU9" t="n">
-        <v>153.4300689655172</v>
+        <v>163.0275862068966</v>
       </c>
       <c r="FV9" t="n">
-        <v>1385.535724137931</v>
+        <v>1569.807448275862</v>
       </c>
       <c r="FW9" t="n">
-        <v>1161.092413793103</v>
+        <v>1309.556137931035</v>
       </c>
       <c r="FX9" t="n">
-        <v>216.6681379310344</v>
+        <v>245.7270344827587</v>
       </c>
       <c r="FY9" t="n">
-        <v>0.3724621734587251</v>
+        <v>0.4985141065830721</v>
       </c>
       <c r="FZ9" t="n">
-        <v>1.105213270637408</v>
+        <v>1.014519936204147</v>
       </c>
       <c r="GA9" t="n">
-        <v>0.5121740558292281</v>
+        <v>0.04940229885057471</v>
       </c>
       <c r="GB9" t="n">
-        <v>1.110177937005523</v>
+        <v>0.7338486938349007</v>
       </c>
       <c r="GC9" t="n">
-        <v>0.09659505923354554</v>
+        <v>0.08894505357302807</v>
       </c>
       <c r="GD9" t="n">
-        <v>0.2879053191503867</v>
+        <v>0.3160173167728403</v>
       </c>
       <c r="GE9" t="n">
-        <v>2.166681379310344</v>
+        <v>2.457270344827586</v>
       </c>
       <c r="GF9" t="n">
-        <v>1.316348891677878</v>
+        <v>1.48284865249276</v>
       </c>
       <c r="GG9" t="n">
-        <v>0.1316998643941555</v>
+        <v>0.1842667556614572</v>
       </c>
       <c r="GH9" t="n">
-        <v>1.36998766339885</v>
+        <v>1.640936599296939</v>
       </c>
       <c r="GI9" t="n">
-        <v>1.364757137250055</v>
+        <v>1.606310855987215</v>
       </c>
       <c r="GJ9" t="n">
-        <v>0.1269113786228383</v>
+        <v>0.1257598474133188</v>
       </c>
       <c r="GK9" t="n">
-        <v>-0.5153103448275855</v>
+        <v>-2.112827586206897</v>
       </c>
       <c r="GL9" t="n">
-        <v>-0.7517241379310278</v>
+        <v>-10.32579310344828</v>
       </c>
       <c r="GM9" t="n">
-        <v>-3.274758620689653</v>
+        <v>-1.595862068965516</v>
       </c>
       <c r="GN9" t="n">
-        <v>21.21186206896553</v>
+        <v>-47.71751724137933</v>
       </c>
       <c r="GO9" t="n">
-        <v>5.812965517241388</v>
+        <v>0.8620689655172384</v>
       </c>
       <c r="GP9" t="n">
-        <v>3.730482758620695</v>
+        <v>-9.358344827586206</v>
       </c>
       <c r="GQ9" t="n">
-        <v>33.84910344827588</v>
+        <v>-7.736275862068965</v>
       </c>
       <c r="GR9" t="n">
-        <v>150.7348965517247</v>
+        <v>-522.3172413793106</v>
       </c>
       <c r="GS9" t="n">
-        <v>11.44910344827587</v>
+        <v>-0.921103448275872</v>
       </c>
       <c r="GT9" t="n">
-        <v>10.13048275862069</v>
+        <v>-8.248551724137936</v>
       </c>
       <c r="GU9" t="n">
-        <v>2.798896551724141</v>
+        <v>4.86013793103448</v>
       </c>
       <c r="GV9" t="n">
-        <v>-2.183448275862048</v>
+        <v>14.7616551724138</v>
       </c>
       <c r="GW9" t="n">
-        <v>4.06593103448276</v>
+        <v>-2.649931034482759</v>
       </c>
       <c r="GX9" t="n">
-        <v>3.385931034482759</v>
+        <v>1.439448275862066</v>
       </c>
       <c r="GY9" t="n">
-        <v>11.1944827586207</v>
+        <v>-4.736551724137939</v>
       </c>
       <c r="GZ9" t="n">
-        <v>32.37903448275864</v>
+        <v>9.919724137931041</v>
       </c>
       <c r="HA9" t="n">
-        <v>117.8838620689658</v>
+        <v>-552.5335172413795</v>
       </c>
       <c r="HB9" t="n">
-        <v>36.07503448275907</v>
+        <v>-530.7561379310346</v>
       </c>
       <c r="HC9" t="n">
-        <v>23.00744827586215</v>
+        <v>-43.23903448275865</v>
       </c>
       <c r="HD9" t="n">
-        <v>-0.01909902473005909</v>
+        <v>-0.1409042038421349</v>
       </c>
       <c r="HE9" t="n">
-        <v>-0.1741197143852313</v>
+        <v>-0.003204640006091886</v>
       </c>
       <c r="HF9" t="n">
-        <v>-0.06550286112355069</v>
+        <v>0.3252816091954023</v>
       </c>
       <c r="HG9" t="n">
-        <v>0.1029794994277755</v>
+        <v>0.0851502919663164</v>
       </c>
       <c r="HH9" t="n">
-        <v>0.07329126290937006</v>
+        <v>0.0225572293422702</v>
       </c>
       <c r="HI9" t="n">
-        <v>0.098829194141618</v>
+        <v>0.1744143915640186</v>
       </c>
       <c r="HJ9" t="n">
-        <v>0.2300744827586216</v>
+        <v>-0.4323903448275863</v>
       </c>
       <c r="HK9" t="n">
-        <v>0.19994334602022</v>
+        <v>-0.2578332994549937</v>
       </c>
       <c r="HL9" t="n">
-        <v>0.0464173162613</v>
+        <v>-0.05309120129749906</v>
       </c>
       <c r="HM9" t="n">
-        <v>0.2211188991571302</v>
+        <v>-0.4710951733572382</v>
       </c>
       <c r="HN9" t="n">
-        <v>0.2106385884288726</v>
+        <v>-0.3820081624155756</v>
       </c>
       <c r="HO9" t="n">
-        <v>0.08194708655126165</v>
+        <v>0.01307190161602673</v>
       </c>
     </row>
     <row r="10">

</xml_diff>